<commit_message>
Atualiza dados SEMANA ATUAL ate quarta-feira (22/07) + regenera cache
</commit_message>
<xml_diff>
--- a/data/SEMANA ATUAL/ELANCO.xlsx
+++ b/data/SEMANA ATUAL/ELANCO.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="275">
   <si>
     <t>Sigla Loja</t>
   </si>
@@ -26,6 +26,9 @@
   </si>
   <si>
     <t>21/07/2026 (Ter)</t>
+  </si>
+  <si>
+    <t>22/07/2026 (Qua)</t>
   </si>
   <si>
     <t>ABNO-RJ</t>
@@ -1201,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D270"/>
+  <dimension ref="A1:E270"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -1209,7 +1212,7 @@
     <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1222,21 +1225,27 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1">
-        <v>445.8799999999999</v>
+        <v>445.88</v>
       </c>
       <c r="D2" s="1">
         <v>1385.85</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2" s="1">
+        <v>1296.09</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1">
         <v>789.45</v>
@@ -1244,21 +1253,27 @@
       <c r="D3" s="1">
         <v>1815.69</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3" s="1">
+        <v>2613.22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="1">
         <v>1958.65</v>
       </c>
       <c r="D4" s="1">
-        <v>1417.78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>1483.77</v>
+      </c>
+      <c r="E4" s="1">
+        <v>3192.27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" s="1">
         <v>801.5999999999999</v>
@@ -1266,10 +1281,13 @@
       <c r="D5" s="1">
         <v>1048.9</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5" s="1">
+        <v>1011.06</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1">
         <v>1147.61</v>
@@ -1277,10 +1295,13 @@
       <c r="D6" s="1">
         <v>696.52</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6" s="1">
+        <v>591.01</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1">
         <v>1157.41</v>
@@ -1288,10 +1309,13 @@
       <c r="D7" s="1">
         <v>1536.43</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7" s="1">
+        <v>1369.74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" s="1">
         <v>390.76</v>
@@ -1299,10 +1323,13 @@
       <c r="D8" s="1">
         <v>1494.81</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8" s="1">
+        <v>695.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="1">
         <v>1785.11</v>
@@ -1310,10 +1337,13 @@
       <c r="D9" s="1">
         <v>443.06</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9" s="1">
+        <v>381.81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" s="1">
         <v>390.86</v>
@@ -1321,10 +1351,13 @@
       <c r="D10" s="1">
         <v>108.98</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10" s="1">
+        <v>167.29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="1">
         <v>1599.09</v>
@@ -1332,32 +1365,41 @@
       <c r="D11" s="1">
         <v>783.3000000000002</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11" s="1">
+        <v>838.0400000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12" s="1">
-        <v>847.8999999999999</v>
+        <v>847.9</v>
       </c>
       <c r="D12" s="1">
         <v>1028.07</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="E12" s="1">
+        <v>219.34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" s="1">
         <v>1563.49</v>
       </c>
       <c r="D13" s="1">
-        <v>865.0500000000002</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
+        <v>865.05</v>
+      </c>
+      <c r="E13" s="1">
+        <v>586.35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="1">
         <v>1765.93</v>
@@ -1365,10 +1407,13 @@
       <c r="D14" s="1">
         <v>1166.09</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="E14" s="1">
+        <v>704.51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C15" s="1">
         <v>2739.02</v>
@@ -1376,21 +1421,27 @@
       <c r="D15" s="1">
         <v>813.97</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="E15" s="1">
+        <v>1495.51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" s="1">
-        <v>343.9499999999999</v>
+        <v>343.95</v>
       </c>
       <c r="D16" s="1">
         <v>122.99</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16" s="1">
+        <v>503.11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C17" s="1">
         <v>254.18</v>
@@ -1398,32 +1449,41 @@
       <c r="D17" s="1">
         <v>642.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17" s="1">
+        <v>1378.28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C18" s="1">
         <v>108.98</v>
       </c>
       <c r="D18" s="1">
-        <v>652.9200000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
+        <v>652.92</v>
+      </c>
+      <c r="E18" s="1">
+        <v>998.8900000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="1">
-        <v>553.1899999999999</v>
+        <v>553.1900000000001</v>
       </c>
       <c r="D19" s="1">
         <v>1415.99</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19" s="1">
+        <v>2140.98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C20" s="1">
         <v>1445.73</v>
@@ -1431,10 +1491,13 @@
       <c r="D20" s="1">
         <v>566.17</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20" s="1">
+        <v>654.64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C21" s="1">
         <v>627.96</v>
@@ -1442,21 +1505,27 @@
       <c r="D21" s="1">
         <v>1020.07</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21" s="1">
+        <v>33.99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C22" s="1">
-        <v>520.84</v>
+        <v>520.8399999999999</v>
       </c>
       <c r="D22" s="1">
         <v>288.97</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22" s="1">
+        <v>249.96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C23" s="1">
         <v>418.6799999999999</v>
@@ -1464,10 +1533,13 @@
       <c r="D23" s="1">
         <v>66.98999999999999</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23" s="1">
+        <v>128.97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C24" s="1">
         <v>1163.73</v>
@@ -1475,10 +1547,13 @@
       <c r="D24" s="1">
         <v>1606.52</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24" s="1">
+        <v>1201.46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C25" s="1">
         <v>54.67</v>
@@ -1486,21 +1561,27 @@
       <c r="D25" s="1">
         <v>97.48999999999999</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25" s="1">
+        <v>1086.88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C26" s="1">
-        <v>2380.559999999999</v>
+        <v>2380.56</v>
       </c>
       <c r="D26" s="1">
         <v>1960.76</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26" s="1">
+        <v>1777.39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C27" s="1">
         <v>1030.88</v>
@@ -1508,10 +1589,13 @@
       <c r="D27" s="1">
         <v>431.06</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="E27" s="1">
+        <v>888.48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C28" s="1">
         <v>1804.99</v>
@@ -1519,10 +1603,13 @@
       <c r="D28" s="1">
         <v>1171.54</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="E28" s="1">
+        <v>2323.24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C29" s="1">
         <v>1723.5</v>
@@ -1530,10 +1617,13 @@
       <c r="D29" s="1">
         <v>3184.79</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="E29" s="1">
+        <v>2849.819999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C30" s="1">
         <v>220.88</v>
@@ -1541,10 +1631,13 @@
       <c r="D30" s="1">
         <v>366.39</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="E30" s="1">
+        <v>1587.96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C31" s="1">
         <v>393.74</v>
@@ -1552,10 +1645,13 @@
       <c r="D31" s="1">
         <v>863.03</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="E31" s="1">
+        <v>1019.53</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C32" s="1">
         <v>1396.49</v>
@@ -1563,10 +1659,13 @@
       <c r="D32" s="1">
         <v>2038.42</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="E32" s="1">
+        <v>1815.82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C33" s="1">
         <v>1989.83</v>
@@ -1574,32 +1673,41 @@
       <c r="D33" s="1">
         <v>2293.22</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="E33" s="1">
+        <v>1648.61</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C34" s="1">
         <v>2000.7</v>
       </c>
       <c r="D34" s="1">
-        <v>2667.030000000001</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
+        <v>2667.03</v>
+      </c>
+      <c r="E34" s="1">
+        <v>2344.08</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C35" s="1">
         <v>395.47</v>
       </c>
       <c r="D35" s="1">
-        <v>837.86</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
+        <v>837.8599999999999</v>
+      </c>
+      <c r="E35" s="1">
+        <v>975.1300000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C36" s="1">
         <v>786.2</v>
@@ -1607,21 +1715,27 @@
       <c r="D36" s="1">
         <v>605.54</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="E36" s="1">
+        <v>582.95</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C37" s="1">
-        <v>2319.15</v>
+        <v>2319.150000000001</v>
       </c>
       <c r="D37" s="1">
         <v>1969.78</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="E37" s="1">
+        <v>1869.32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C38" s="1">
         <v>520.28</v>
@@ -1629,10 +1743,13 @@
       <c r="D38" s="1">
         <v>593.25</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="E38" s="1">
+        <v>169.75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C39" s="1">
         <v>889.1600000000001</v>
@@ -1640,10 +1757,13 @@
       <c r="D39" s="1">
         <v>452.16</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39" s="1">
+        <v>646.53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C40" s="1">
         <v>678.58</v>
@@ -1651,10 +1771,13 @@
       <c r="D40" s="1">
         <v>137.23</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="E40" s="1">
+        <v>1957.65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C41" s="1">
         <v>1482.7</v>
@@ -1662,43 +1785,55 @@
       <c r="D41" s="1">
         <v>52.5</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="E41" s="1">
+        <v>734.36</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C42" s="1">
-        <v>662.0899999999999</v>
+        <v>662.09</v>
       </c>
       <c r="D42" s="1">
         <v>760.05</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="E42" s="1">
+        <v>1497.61</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C43" s="1">
         <v>603.41</v>
       </c>
       <c r="D43" s="1">
-        <v>957.3200000000001</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
+        <v>957.3200000000002</v>
+      </c>
+      <c r="E43" s="1">
+        <v>124.99</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C44" s="1">
-        <v>932.46</v>
+        <v>932.4599999999999</v>
       </c>
       <c r="D44" s="1">
         <v>1355.41</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="E44" s="1">
+        <v>1389.05</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C45" s="1">
         <v>1474.12</v>
@@ -1706,10 +1841,13 @@
       <c r="D45" s="1">
         <v>1052.33</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="E45" s="1">
+        <v>1352.11</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C46" s="1">
         <v>2230.79</v>
@@ -1717,10 +1855,13 @@
       <c r="D46" s="1">
         <v>1243.55</v>
       </c>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="E46" s="1">
+        <v>1144.73</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C47" s="1">
         <v>798.9400000000001</v>
@@ -1728,10 +1869,13 @@
       <c r="D47" s="1">
         <v>971.9200000000001</v>
       </c>
-    </row>
-    <row r="48" spans="1:4">
+      <c r="E47" s="1">
+        <v>676.92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C48" s="1">
         <v>2239.55</v>
@@ -1739,10 +1883,13 @@
       <c r="D48" s="1">
         <v>1597.49</v>
       </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="E48" s="1">
+        <v>1975.56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C49" s="1">
         <v>2078.41</v>
@@ -1750,21 +1897,27 @@
       <c r="D49" s="1">
         <v>1485.55</v>
       </c>
-    </row>
-    <row r="50" spans="1:4">
+      <c r="E49" s="1">
+        <v>1318.86</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C50" s="1">
         <v>670.9299999999999</v>
       </c>
       <c r="D50" s="1">
-        <v>452.9000000000001</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4">
+        <v>452.9</v>
+      </c>
+      <c r="E50" s="1">
+        <v>91.98999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C51" s="1">
         <v>1101.94</v>
@@ -1772,21 +1925,27 @@
       <c r="D51" s="1">
         <v>1117.38</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="E51" s="1">
+        <v>1083.94</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D52" s="1">
         <v>592.76</v>
       </c>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="E52" s="1">
+        <v>670.74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C53" s="1">
         <v>358.96</v>
@@ -1794,10 +1953,13 @@
       <c r="D53" s="1">
         <v>723.1</v>
       </c>
-    </row>
-    <row r="54" spans="1:4">
+      <c r="E53" s="1">
+        <v>247.77</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C54" s="1">
         <v>64.98999999999999</v>
@@ -1805,21 +1967,27 @@
       <c r="D54" s="1">
         <v>261.97</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
+      <c r="E54" s="1">
+        <v>50.99</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C55" s="1">
         <v>327.89</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4">
+        <v>56</v>
+      </c>
+      <c r="E55" s="1">
+        <v>273.24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C56" s="1">
         <v>266.04</v>
@@ -1827,32 +1995,41 @@
       <c r="D56" s="1">
         <v>398.98</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="E56" s="1">
+        <v>248.79</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C57" s="1">
-        <v>5368.460000000001</v>
+        <v>5368.46</v>
       </c>
       <c r="D57" s="1">
-        <v>4112.700000000001</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4">
+        <v>4112.7</v>
+      </c>
+      <c r="E57" s="1">
+        <v>3414.81</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C58" s="1">
         <v>808.5</v>
       </c>
       <c r="D58" s="1">
-        <v>960.1099999999999</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4">
+        <v>960.1100000000001</v>
+      </c>
+      <c r="E58" s="1">
+        <v>643.45</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C59" s="1">
         <v>453.9399999999999</v>
@@ -1860,10 +2037,13 @@
       <c r="D59" s="1">
         <v>763.46</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="E59" s="1">
+        <v>943.96</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C60" s="1">
         <v>253.29</v>
@@ -1871,10 +2051,13 @@
       <c r="D60" s="1">
         <v>278.97</v>
       </c>
-    </row>
-    <row r="61" spans="1:4">
+      <c r="E60" s="1">
+        <v>1198.75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C61" s="1">
         <v>857.42</v>
@@ -1882,10 +2065,13 @@
       <c r="D61" s="1">
         <v>1149.13</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
+      <c r="E61" s="1">
+        <v>2554.33</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C62" s="1">
         <v>156.72</v>
@@ -1893,21 +2079,27 @@
       <c r="D62" s="1">
         <v>79.98999999999999</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
+      <c r="E62" s="1">
+        <v>210.32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C63" s="1">
         <v>1024.83</v>
       </c>
       <c r="D63" s="1">
-        <v>929.41</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4">
+        <v>929.4100000000001</v>
+      </c>
+      <c r="E63" s="1">
+        <v>982.5799999999999</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C64" s="1">
         <v>688.65</v>
@@ -1915,10 +2107,13 @@
       <c r="D64" s="1">
         <v>1109.4</v>
       </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="E64" s="1">
+        <v>141.98</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C65" s="1">
         <v>446.4</v>
@@ -1926,21 +2121,27 @@
       <c r="D65" s="1">
         <v>212.97</v>
       </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="E65" s="1">
+        <v>64.98999999999999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C66" s="1">
-        <v>743.9100000000001</v>
+        <v>743.91</v>
       </c>
       <c r="D66" s="1">
         <v>607</v>
       </c>
-    </row>
-    <row r="67" spans="1:4">
+      <c r="E66" s="1">
+        <v>1004.62</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C67" s="1">
         <v>945.45</v>
@@ -1948,10 +2149,13 @@
       <c r="D67" s="1">
         <v>1229.38</v>
       </c>
-    </row>
-    <row r="68" spans="1:4">
+      <c r="E67" s="1">
+        <v>784.62</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C68" s="1">
         <v>513.95</v>
@@ -1959,10 +2163,13 @@
       <c r="D68" s="1">
         <v>840.26</v>
       </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="E68" s="1">
+        <v>262.19</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C69" s="1">
         <v>202.08</v>
@@ -1970,10 +2177,13 @@
       <c r="D69" s="1">
         <v>485.23</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="E69" s="1">
+        <v>1093.61</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C70" s="1">
         <v>1267.93</v>
@@ -1981,10 +2191,13 @@
       <c r="D70" s="1">
         <v>1167.2</v>
       </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="E70" s="1">
+        <v>323.37</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C71" s="1">
         <v>668.09</v>
@@ -1992,10 +2205,13 @@
       <c r="D71" s="1">
         <v>557.77</v>
       </c>
-    </row>
-    <row r="72" spans="1:4">
+      <c r="E71" s="1">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C72" s="1">
         <v>1081.36</v>
@@ -2003,10 +2219,13 @@
       <c r="D72" s="1">
         <v>423.32</v>
       </c>
-    </row>
-    <row r="73" spans="1:4">
+      <c r="E72" s="1">
+        <v>656.46</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C73" s="1">
         <v>188.72</v>
@@ -2014,21 +2233,27 @@
       <c r="D73" s="1">
         <v>1758.8</v>
       </c>
-    </row>
-    <row r="74" spans="1:4">
+      <c r="E73" s="1">
+        <v>1525.28</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C74" s="1">
-        <v>450.93</v>
+        <v>450.9299999999999</v>
       </c>
       <c r="D74" s="1">
         <v>673.9400000000001</v>
       </c>
-    </row>
-    <row r="75" spans="1:4">
+      <c r="E74" s="1">
+        <v>517.4400000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C75" s="1">
         <v>64.98999999999999</v>
@@ -2036,10 +2261,13 @@
       <c r="D75" s="1">
         <v>329.56</v>
       </c>
-    </row>
-    <row r="76" spans="1:4">
+      <c r="E75" s="1">
+        <v>191.25</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C76" s="1">
         <v>2642.34</v>
@@ -2047,10 +2275,13 @@
       <c r="D76" s="1">
         <v>1508.66</v>
       </c>
-    </row>
-    <row r="77" spans="1:4">
+      <c r="E76" s="1">
+        <v>2137.01</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C77" s="1">
         <v>1699.59</v>
@@ -2058,10 +2289,13 @@
       <c r="D77" s="1">
         <v>2399.88</v>
       </c>
-    </row>
-    <row r="78" spans="1:4">
+      <c r="E77" s="1">
+        <v>2282.78</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C78" s="1">
         <v>36.99</v>
@@ -2069,10 +2303,13 @@
       <c r="D78" s="1">
         <v>1229.42</v>
       </c>
-    </row>
-    <row r="79" spans="1:4">
+      <c r="E78" s="1">
+        <v>279.12</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C79" s="1">
         <v>1059.71</v>
@@ -2080,10 +2317,13 @@
       <c r="D79" s="1">
         <v>490.43</v>
       </c>
-    </row>
-    <row r="80" spans="1:4">
+      <c r="E79" s="1">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C80" s="1">
         <v>511.27</v>
@@ -2091,10 +2331,13 @@
       <c r="D80" s="1">
         <v>866.0200000000001</v>
       </c>
-    </row>
-    <row r="81" spans="1:4">
+      <c r="E80" s="1">
+        <v>164.95</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C81" s="1">
         <v>343.82</v>
@@ -2102,10 +2345,13 @@
       <c r="D81" s="1">
         <v>747.58</v>
       </c>
-    </row>
-    <row r="82" spans="1:4">
+      <c r="E81" s="1">
+        <v>150.84</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C82" s="1">
         <v>523.5700000000001</v>
@@ -2113,10 +2359,13 @@
       <c r="D82" s="1">
         <v>628.66</v>
       </c>
-    </row>
-    <row r="83" spans="1:4">
+      <c r="E82" s="1">
+        <v>200.64</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C83" s="1">
         <v>566.77</v>
@@ -2124,10 +2373,13 @@
       <c r="D83" s="1">
         <v>669.3099999999999</v>
       </c>
-    </row>
-    <row r="84" spans="1:4">
+      <c r="E83" s="1">
+        <v>275.41</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C84" s="1">
         <v>630.76</v>
@@ -2135,21 +2387,27 @@
       <c r="D84" s="1">
         <v>1071.75</v>
       </c>
-    </row>
-    <row r="85" spans="1:4">
+      <c r="E84" s="1">
+        <v>400.94</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C85" s="1">
-        <v>3378.69</v>
+        <v>3378.689999999999</v>
       </c>
       <c r="D85" s="1">
-        <v>2575.24</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4">
+        <v>2575.239999999999</v>
+      </c>
+      <c r="E85" s="1">
+        <v>3203.239999999999</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
       <c r="A86" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C86" s="1">
         <v>395.98</v>
@@ -2157,10 +2415,13 @@
       <c r="D86" s="1">
         <v>251.64</v>
       </c>
-    </row>
-    <row r="87" spans="1:4">
+      <c r="E86" s="1">
+        <v>278.63</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C87" s="1">
         <v>33.99</v>
@@ -2168,21 +2429,27 @@
       <c r="D87" s="1">
         <v>177.19</v>
       </c>
-    </row>
-    <row r="88" spans="1:4">
+      <c r="E87" s="1">
+        <v>429.54</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C88" s="1">
-        <v>683.79</v>
+        <v>683.7900000000001</v>
       </c>
       <c r="D88" s="1">
         <v>390.9</v>
       </c>
-    </row>
-    <row r="89" spans="1:4">
+      <c r="E88" s="1">
+        <v>515.26</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C89" s="1">
         <v>97.98999999999999</v>
@@ -2190,10 +2457,13 @@
       <c r="D89" s="1">
         <v>191.22</v>
       </c>
-    </row>
-    <row r="90" spans="1:4">
+      <c r="E89" s="1">
+        <v>370.04</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C90" s="1">
         <v>1703.16</v>
@@ -2201,21 +2471,27 @@
       <c r="D90" s="1">
         <v>2122.54</v>
       </c>
-    </row>
-    <row r="91" spans="1:4">
+      <c r="E90" s="1">
+        <v>1288.45</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C91" s="1">
-        <v>966.54</v>
+        <v>966.5400000000001</v>
       </c>
       <c r="D91" s="1">
         <v>315.96</v>
       </c>
-    </row>
-    <row r="92" spans="1:4">
+      <c r="E91" s="1">
+        <v>364.02</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C92" s="1">
         <v>1454.25</v>
@@ -2223,10 +2499,13 @@
       <c r="D92" s="1">
         <v>1613.3</v>
       </c>
-    </row>
-    <row r="93" spans="1:4">
+      <c r="E92" s="1">
+        <v>730.9400000000001</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C93" s="1">
         <v>137.75</v>
@@ -2234,10 +2513,13 @@
       <c r="D93" s="1">
         <v>1140.52</v>
       </c>
-    </row>
-    <row r="94" spans="1:4">
+      <c r="E93" s="1">
+        <v>563.22</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C94" s="1">
         <v>1202.53</v>
@@ -2245,10 +2527,13 @@
       <c r="D94" s="1">
         <v>1597.1</v>
       </c>
-    </row>
-    <row r="95" spans="1:4">
+      <c r="E94" s="1">
+        <v>2236.03</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C95" s="1">
         <v>1364.69</v>
@@ -2256,10 +2541,13 @@
       <c r="D95" s="1">
         <v>1663.36</v>
       </c>
-    </row>
-    <row r="96" spans="1:4">
+      <c r="E95" s="1">
+        <v>1568.62</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C96" s="1">
         <v>1560.41</v>
@@ -2267,10 +2555,13 @@
       <c r="D96" s="1">
         <v>425.27</v>
       </c>
-    </row>
-    <row r="97" spans="1:4">
+      <c r="E96" s="1">
+        <v>1704.3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C97" s="1">
         <v>596.5</v>
@@ -2278,10 +2569,13 @@
       <c r="D97" s="1">
         <v>1418.12</v>
       </c>
-    </row>
-    <row r="98" spans="1:4">
+      <c r="E97" s="1">
+        <v>447.2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C98" s="1">
         <v>599.9299999999999</v>
@@ -2289,21 +2583,27 @@
       <c r="D98" s="1">
         <v>550.76</v>
       </c>
-    </row>
-    <row r="99" spans="1:4">
+      <c r="E98" s="1">
+        <v>339.14</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C99" s="1">
-        <v>710.41</v>
+        <v>710.4100000000001</v>
       </c>
       <c r="D99" s="1">
         <v>698.6500000000001</v>
       </c>
-    </row>
-    <row r="100" spans="1:4">
+      <c r="E99" s="1">
+        <v>886.47</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C100" s="1">
         <v>716.23</v>
@@ -2311,10 +2611,13 @@
       <c r="D100" s="1">
         <v>506.2</v>
       </c>
-    </row>
-    <row r="101" spans="1:4">
+      <c r="E100" s="1">
+        <v>842.5599999999999</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C101" s="1">
         <v>902.17</v>
@@ -2322,10 +2625,13 @@
       <c r="D101" s="1">
         <v>955.2400000000001</v>
       </c>
-    </row>
-    <row r="102" spans="1:4">
+      <c r="E101" s="1">
+        <v>1038.64</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C102" s="1">
         <v>1033.94</v>
@@ -2333,21 +2639,27 @@
       <c r="D102" s="1">
         <v>1051.22</v>
       </c>
-    </row>
-    <row r="103" spans="1:4">
+      <c r="E102" s="1">
+        <v>227.92</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C103" s="1">
-        <v>769.26</v>
+        <v>769.2600000000001</v>
       </c>
       <c r="D103" s="1">
         <v>483.86</v>
       </c>
-    </row>
-    <row r="104" spans="1:4">
+      <c r="E103" s="1">
+        <v>289.91</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C104" s="1">
         <v>259.97</v>
@@ -2355,10 +2667,13 @@
       <c r="D104" s="1">
         <v>394.47</v>
       </c>
-    </row>
-    <row r="105" spans="1:4">
+      <c r="E104" s="1">
+        <v>427.87</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C105" s="1">
         <v>1637.22</v>
@@ -2366,21 +2681,27 @@
       <c r="D105" s="1">
         <v>55.19</v>
       </c>
-    </row>
-    <row r="106" spans="1:4">
+      <c r="E105" s="1">
+        <v>778.6300000000001</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C106" s="1">
         <v>1251.47</v>
       </c>
       <c r="D106" s="1">
-        <v>365.18</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4">
+        <v>365.1799999999999</v>
+      </c>
+      <c r="E106" s="1">
+        <v>966.33</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C107" s="1">
         <v>1141.94</v>
@@ -2388,43 +2709,55 @@
       <c r="D107" s="1">
         <v>450.29</v>
       </c>
-    </row>
-    <row r="108" spans="1:4">
+      <c r="E107" s="1">
+        <v>1437.08</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C108" s="1">
-        <v>635.5400000000001</v>
+        <v>635.54</v>
       </c>
       <c r="D108" s="1">
         <v>886.8099999999999</v>
       </c>
-    </row>
-    <row r="109" spans="1:4">
+      <c r="E108" s="1">
+        <v>558.51</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5">
       <c r="A109" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C109" s="1">
         <v>1150.98</v>
       </c>
       <c r="D109" s="1">
-        <v>545.9200000000001</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4">
+        <v>545.92</v>
+      </c>
+      <c r="E109" s="1">
+        <v>690.76</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C110" s="1">
         <v>709.96</v>
       </c>
       <c r="D110" s="1">
-        <v>556.96</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4">
+        <v>556.9599999999999</v>
+      </c>
+      <c r="E110" s="1">
+        <v>108.73</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C111" s="1">
         <v>166.4</v>
@@ -2432,10 +2765,13 @@
       <c r="D111" s="1">
         <v>104.98</v>
       </c>
-    </row>
-    <row r="112" spans="1:4">
+      <c r="E111" s="1">
+        <v>241.98</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C112" s="1">
         <v>782.91</v>
@@ -2443,10 +2779,13 @@
       <c r="D112" s="1">
         <v>260.85</v>
       </c>
-    </row>
-    <row r="113" spans="1:4">
+      <c r="E112" s="1">
+        <v>720.77</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C113" s="1">
         <v>1289.72</v>
@@ -2454,21 +2793,27 @@
       <c r="D113" s="1">
         <v>594.1</v>
       </c>
-    </row>
-    <row r="114" spans="1:4">
+      <c r="E113" s="1">
+        <v>580.4</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C114" s="1">
         <v>64.48999999999999</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4">
+        <v>56</v>
+      </c>
+      <c r="E114" s="1">
+        <v>376.98</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C115" s="1">
         <v>454.96</v>
@@ -2476,10 +2821,13 @@
       <c r="D115" s="1">
         <v>709.4000000000001</v>
       </c>
-    </row>
-    <row r="116" spans="1:4">
+      <c r="E115" s="1">
+        <v>197.49</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C116" s="1">
         <v>207.55</v>
@@ -2487,10 +2835,13 @@
       <c r="D116" s="1">
         <v>443.07</v>
       </c>
-    </row>
-    <row r="117" spans="1:4">
+      <c r="E116" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C117" s="1">
         <v>1188.89</v>
@@ -2498,10 +2849,13 @@
       <c r="D117" s="1">
         <v>956.24</v>
       </c>
-    </row>
-    <row r="118" spans="1:4">
+      <c r="E117" s="1">
+        <v>1143.63</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C118" s="1">
         <v>608.3099999999999</v>
@@ -2509,10 +2863,13 @@
       <c r="D118" s="1">
         <v>1027.95</v>
       </c>
-    </row>
-    <row r="119" spans="1:4">
+      <c r="E118" s="1">
+        <v>724.96</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C119" s="1">
         <v>1487.89</v>
@@ -2520,10 +2877,13 @@
       <c r="D119" s="1">
         <v>2163.309999999999</v>
       </c>
-    </row>
-    <row r="120" spans="1:4">
+      <c r="E119" s="1">
+        <v>1670.22</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C120" s="1">
         <v>971.9299999999999</v>
@@ -2531,10 +2891,13 @@
       <c r="D120" s="1">
         <v>42.99</v>
       </c>
-    </row>
-    <row r="121" spans="1:4">
+      <c r="E120" s="1">
+        <v>103.64</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C121" s="1">
         <v>700.6900000000001</v>
@@ -2542,10 +2905,13 @@
       <c r="D121" s="1">
         <v>1097.58</v>
       </c>
-    </row>
-    <row r="122" spans="1:4">
+      <c r="E121" s="1">
+        <v>454.19</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C122" s="1">
         <v>1206.27</v>
@@ -2553,10 +2919,13 @@
       <c r="D122" s="1">
         <v>2100.63</v>
       </c>
-    </row>
-    <row r="123" spans="1:4">
+      <c r="E122" s="1">
+        <v>468.35</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C123" s="1">
         <v>910.9400000000001</v>
@@ -2564,10 +2933,13 @@
       <c r="D123" s="1">
         <v>391.61</v>
       </c>
-    </row>
-    <row r="124" spans="1:4">
+      <c r="E123" s="1">
+        <v>948.97</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C124" s="1">
         <v>105.99</v>
@@ -2575,10 +2947,13 @@
       <c r="D124" s="1">
         <v>144.97</v>
       </c>
-    </row>
-    <row r="125" spans="1:4">
+      <c r="E124" s="1">
+        <v>512.42</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C125" s="1">
         <v>271.98</v>
@@ -2586,10 +2961,13 @@
       <c r="D125" s="1">
         <v>670.78</v>
       </c>
-    </row>
-    <row r="126" spans="1:4">
+      <c r="E125" s="1">
+        <v>399.22</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C126" s="1">
         <v>668.51</v>
@@ -2597,10 +2975,13 @@
       <c r="D126" s="1">
         <v>1266.67</v>
       </c>
-    </row>
-    <row r="127" spans="1:4">
+      <c r="E126" s="1">
+        <v>1213.85</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C127" s="1">
         <v>1092.61</v>
@@ -2608,10 +2989,13 @@
       <c r="D127" s="1">
         <v>404.26</v>
       </c>
-    </row>
-    <row r="128" spans="1:4">
+      <c r="E127" s="1">
+        <v>1093.25</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C128" s="1">
         <v>851.95</v>
@@ -2619,32 +3003,41 @@
       <c r="D128" s="1">
         <v>571.9</v>
       </c>
-    </row>
-    <row r="129" spans="1:4">
+      <c r="E128" s="1">
+        <v>148.39</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C129" s="1">
-        <v>703.7400000000001</v>
+        <v>703.74</v>
       </c>
       <c r="D129" s="1">
         <v>247.66</v>
       </c>
-    </row>
-    <row r="130" spans="1:4">
+      <c r="E129" s="1">
+        <v>1249.18</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C130" s="1">
-        <v>925.02</v>
+        <v>925.0200000000001</v>
       </c>
       <c r="D130" s="1">
         <v>1399.18</v>
       </c>
-    </row>
-    <row r="131" spans="1:4">
+      <c r="E130" s="1">
+        <v>1737.35</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5">
       <c r="A131" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C131" s="1">
         <v>286.21</v>
@@ -2652,10 +3045,13 @@
       <c r="D131" s="1">
         <v>39.99</v>
       </c>
-    </row>
-    <row r="132" spans="1:4">
+      <c r="E131" s="1">
+        <v>131.6</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C132" s="1">
         <v>967.87</v>
@@ -2663,10 +3059,13 @@
       <c r="D132" s="1">
         <v>812.33</v>
       </c>
-    </row>
-    <row r="133" spans="1:4">
+      <c r="E132" s="1">
+        <v>1185.79</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C133" s="1">
         <v>1878.23</v>
@@ -2674,21 +3073,27 @@
       <c r="D133" s="1">
         <v>1543.28</v>
       </c>
-    </row>
-    <row r="134" spans="1:4">
+      <c r="E133" s="1">
+        <v>1368.94</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C134" s="1">
-        <v>751.1600000000001</v>
+        <v>751.16</v>
       </c>
       <c r="D134" s="1">
         <v>468.96</v>
       </c>
-    </row>
-    <row r="135" spans="1:4">
+      <c r="E134" s="1">
+        <v>820.34</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C135" s="1">
         <v>1315.46</v>
@@ -2696,10 +3101,13 @@
       <c r="D135" s="1">
         <v>764.1500000000001</v>
       </c>
-    </row>
-    <row r="136" spans="1:4">
+      <c r="E135" s="1">
+        <v>1042.97</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C136" s="1">
         <v>128.98</v>
@@ -2707,10 +3115,13 @@
       <c r="D136" s="1">
         <v>184.84</v>
       </c>
-    </row>
-    <row r="137" spans="1:4">
+      <c r="E136" s="1">
+        <v>42.99</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C137" s="1">
         <v>1027.34</v>
@@ -2718,10 +3129,13 @@
       <c r="D137" s="1">
         <v>1846.03</v>
       </c>
-    </row>
-    <row r="138" spans="1:4">
+      <c r="E137" s="1">
+        <v>1204.07</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C138" s="1">
         <v>284.96</v>
@@ -2729,21 +3143,27 @@
       <c r="D138" s="1">
         <v>277.4</v>
       </c>
-    </row>
-    <row r="139" spans="1:4">
+      <c r="E138" s="1">
+        <v>1131.96</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C139" s="1">
-        <v>900.27</v>
+        <v>900.2700000000001</v>
       </c>
       <c r="D139" s="1">
         <v>631.51</v>
       </c>
-    </row>
-    <row r="140" spans="1:4">
+      <c r="E139" s="1">
+        <v>308.66</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C140" s="1">
         <v>601.65</v>
@@ -2751,10 +3171,13 @@
       <c r="D140" s="1">
         <v>409.79</v>
       </c>
-    </row>
-    <row r="141" spans="1:4">
+      <c r="E140" s="1">
+        <v>308.97</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C141" s="1">
         <v>179.99</v>
@@ -2762,10 +3185,13 @@
       <c r="D141" s="1">
         <v>1273.62</v>
       </c>
-    </row>
-    <row r="142" spans="1:4">
+      <c r="E141" s="1">
+        <v>290.99</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C142" s="1">
         <v>680.25</v>
@@ -2773,10 +3199,13 @@
       <c r="D142" s="1">
         <v>425.56</v>
       </c>
-    </row>
-    <row r="143" spans="1:4">
+      <c r="E142" s="1">
+        <v>357.3199999999999</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C143" s="1">
         <v>150.38</v>
@@ -2784,10 +3213,13 @@
       <c r="D143" s="1">
         <v>759.13</v>
       </c>
-    </row>
-    <row r="144" spans="1:4">
+      <c r="E143" s="1">
+        <v>770.55</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5">
       <c r="A144" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C144" s="1">
         <v>191.67</v>
@@ -2795,21 +3227,27 @@
       <c r="D144" s="1">
         <v>170.98</v>
       </c>
-    </row>
-    <row r="145" spans="1:4">
+      <c r="E144" s="1">
+        <v>2102</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C145" s="1">
-        <v>484.94</v>
+        <v>484.9399999999999</v>
       </c>
       <c r="D145" s="1">
         <v>398.97</v>
       </c>
-    </row>
-    <row r="146" spans="1:4">
+      <c r="E145" s="1">
+        <v>511.96</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C146" s="1">
         <v>570.6</v>
@@ -2817,10 +3255,13 @@
       <c r="D146" s="1">
         <v>831.4299999999999</v>
       </c>
-    </row>
-    <row r="147" spans="1:4">
+      <c r="E146" s="1">
+        <v>379.43</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5">
       <c r="A147" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C147" s="1">
         <v>1123.3</v>
@@ -2828,10 +3269,13 @@
       <c r="D147" s="1">
         <v>589.1600000000001</v>
       </c>
-    </row>
-    <row r="148" spans="1:4">
+      <c r="E147" s="1">
+        <v>595.5</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C148" s="1">
         <v>761.24</v>
@@ -2839,10 +3283,13 @@
       <c r="D148" s="1">
         <v>444.59</v>
       </c>
-    </row>
-    <row r="149" spans="1:4">
+      <c r="E148" s="1">
+        <v>1422.24</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5">
       <c r="A149" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C149" s="1">
         <v>1455.54</v>
@@ -2850,10 +3297,13 @@
       <c r="D149" s="1">
         <v>1269.01</v>
       </c>
-    </row>
-    <row r="150" spans="1:4">
+      <c r="E149" s="1">
+        <v>3031.75</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C150" s="1">
         <v>606.96</v>
@@ -2861,32 +3311,41 @@
       <c r="D150" s="1">
         <v>61.27</v>
       </c>
-    </row>
-    <row r="151" spans="1:4">
+      <c r="E150" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C151" s="1">
-        <v>2563.429999999999</v>
+        <v>2563.43</v>
       </c>
       <c r="D151" s="1">
         <v>1664.13</v>
       </c>
-    </row>
-    <row r="152" spans="1:4">
+      <c r="E151" s="1">
+        <v>963.92</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C152" s="1">
-        <v>988.3499999999999</v>
+        <v>988.35</v>
       </c>
       <c r="D152" s="1">
         <v>689.9299999999999</v>
       </c>
-    </row>
-    <row r="153" spans="1:4">
+      <c r="E152" s="1">
+        <v>392.47</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C153" s="1">
         <v>1162.11</v>
@@ -2894,21 +3353,27 @@
       <c r="D153" s="1">
         <v>409.3</v>
       </c>
-    </row>
-    <row r="154" spans="1:4">
+      <c r="E153" s="1">
+        <v>152.39</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C154" s="1">
         <v>1478.7</v>
       </c>
       <c r="D154" s="1">
-        <v>908.3800000000001</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4">
+        <v>908.38</v>
+      </c>
+      <c r="E154" s="1">
+        <v>589.98</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C155" s="1">
         <v>1499.14</v>
@@ -2916,10 +3381,13 @@
       <c r="D155" s="1">
         <v>1889.55</v>
       </c>
-    </row>
-    <row r="156" spans="1:4">
+      <c r="E155" s="1">
+        <v>3340.88</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C156" s="1">
         <v>1383.83</v>
@@ -2927,10 +3395,13 @@
       <c r="D156" s="1">
         <v>418.06</v>
       </c>
-    </row>
-    <row r="157" spans="1:4">
+      <c r="E156" s="1">
+        <v>1526.47</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C157" s="1">
         <v>2027.84</v>
@@ -2938,10 +3409,13 @@
       <c r="D157" s="1">
         <v>129.75</v>
       </c>
-    </row>
-    <row r="158" spans="1:4">
+      <c r="E157" s="1">
+        <v>630.16</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C158" s="1">
         <v>1003.3</v>
@@ -2949,10 +3423,13 @@
       <c r="D158" s="1">
         <v>1330.37</v>
       </c>
-    </row>
-    <row r="159" spans="1:4">
+      <c r="E158" s="1">
+        <v>232.83</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C159" s="1">
         <v>1237.7</v>
@@ -2960,10 +3437,13 @@
       <c r="D159" s="1">
         <v>918.2400000000001</v>
       </c>
-    </row>
-    <row r="160" spans="1:4">
+      <c r="E159" s="1">
+        <v>870.9499999999998</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C160" s="1">
         <v>299.98</v>
@@ -2971,10 +3451,13 @@
       <c r="D160" s="1">
         <v>1545.83</v>
       </c>
-    </row>
-    <row r="161" spans="1:4">
+      <c r="E160" s="1">
+        <v>427.88</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C161" s="1">
         <v>1246.16</v>
@@ -2982,21 +3465,27 @@
       <c r="D161" s="1">
         <v>1794.96</v>
       </c>
-    </row>
-    <row r="162" spans="1:4">
+      <c r="E161" s="1">
+        <v>855.99</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C162" s="1">
         <v>508.96</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4">
+        <v>56</v>
+      </c>
+      <c r="E162" s="1">
+        <v>559.38</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5">
       <c r="A163" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C163" s="1">
         <v>526.45</v>
@@ -3004,10 +3493,13 @@
       <c r="D163" s="1">
         <v>251.23</v>
       </c>
-    </row>
-    <row r="164" spans="1:4">
+      <c r="E163" s="1">
+        <v>341.96</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5">
       <c r="A164" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C164" s="1">
         <v>637.8499999999999</v>
@@ -3015,10 +3507,13 @@
       <c r="D164" s="1">
         <v>68.98999999999999</v>
       </c>
-    </row>
-    <row r="165" spans="1:4">
+      <c r="E164" s="1">
+        <v>334.96</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C165" s="1">
         <v>979.27</v>
@@ -3026,10 +3521,13 @@
       <c r="D165" s="1">
         <v>1874.83</v>
       </c>
-    </row>
-    <row r="166" spans="1:4">
+      <c r="E165" s="1">
+        <v>2692.44</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C166" s="1">
         <v>42.99</v>
@@ -3037,21 +3535,27 @@
       <c r="D166" s="1">
         <v>662.8099999999999</v>
       </c>
-    </row>
-    <row r="167" spans="1:4">
+      <c r="E166" s="1">
+        <v>391.48</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C167" s="1">
         <v>3326.85</v>
       </c>
       <c r="D167" s="1">
-        <v>2899.859999999999</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4">
+        <v>2899.86</v>
+      </c>
+      <c r="E167" s="1">
+        <v>3571.82</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C168" s="1">
         <v>27.19</v>
@@ -3059,10 +3563,13 @@
       <c r="D168" s="1">
         <v>204.99</v>
       </c>
-    </row>
-    <row r="169" spans="1:4">
+      <c r="E168" s="1">
+        <v>452.78</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C169" s="1">
         <v>2564.26</v>
@@ -3070,21 +3577,27 @@
       <c r="D169" s="1">
         <v>1761.91</v>
       </c>
-    </row>
-    <row r="170" spans="1:4">
+      <c r="E169" s="1">
+        <v>1059.56</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D170" s="1">
         <v>336.79</v>
       </c>
-    </row>
-    <row r="171" spans="1:4">
+      <c r="E170" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C171" s="1">
         <v>492.63</v>
@@ -3092,10 +3605,13 @@
       <c r="D171" s="1">
         <v>515.77</v>
       </c>
-    </row>
-    <row r="172" spans="1:4">
+      <c r="E171" s="1">
+        <v>515.6400000000001</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C172" s="1">
         <v>1206.03</v>
@@ -3103,10 +3619,13 @@
       <c r="D172" s="1">
         <v>1519.24</v>
       </c>
-    </row>
-    <row r="173" spans="1:4">
+      <c r="E172" s="1">
+        <v>1446.32</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C173" s="1">
         <v>1347.25</v>
@@ -3114,10 +3633,13 @@
       <c r="D173" s="1">
         <v>1062.41</v>
       </c>
-    </row>
-    <row r="174" spans="1:4">
+      <c r="E173" s="1">
+        <v>1014.16</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C174" s="1">
         <v>2584.34</v>
@@ -3125,10 +3647,13 @@
       <c r="D174" s="1">
         <v>612.63</v>
       </c>
-    </row>
-    <row r="175" spans="1:4">
+      <c r="E174" s="1">
+        <v>773.85</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C175" s="1">
         <v>1081.05</v>
@@ -3136,21 +3661,27 @@
       <c r="D175" s="1">
         <v>1717.27</v>
       </c>
-    </row>
-    <row r="176" spans="1:4">
+      <c r="E175" s="1">
+        <v>1613.29</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C176" s="1">
         <v>739.9400000000001</v>
       </c>
       <c r="D176" s="1">
-        <v>834.9100000000001</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4">
+        <v>834.91</v>
+      </c>
+      <c r="E176" s="1">
+        <v>183.96</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C177" s="1">
         <v>457.68</v>
@@ -3158,10 +3689,13 @@
       <c r="D177" s="1">
         <v>834.9200000000001</v>
       </c>
-    </row>
-    <row r="178" spans="1:4">
+      <c r="E177" s="1">
+        <v>468.9299999999999</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C178" s="1">
         <v>899.9200000000001</v>
@@ -3169,10 +3703,13 @@
       <c r="D178" s="1">
         <v>741.72</v>
       </c>
-    </row>
-    <row r="179" spans="1:4">
+      <c r="E178" s="1">
+        <v>677.4299999999999</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C179" s="1">
         <v>468.21</v>
@@ -3180,10 +3717,13 @@
       <c r="D179" s="1">
         <v>782.84</v>
       </c>
-    </row>
-    <row r="180" spans="1:4">
+      <c r="E179" s="1">
+        <v>431.78</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C180" s="1">
         <v>460.88</v>
@@ -3191,10 +3731,13 @@
       <c r="D180" s="1">
         <v>213.38</v>
       </c>
-    </row>
-    <row r="181" spans="1:4">
+      <c r="E180" s="1">
+        <v>245.98</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C181" s="1">
         <v>381.7</v>
@@ -3202,10 +3745,13 @@
       <c r="D181" s="1">
         <v>53.06</v>
       </c>
-    </row>
-    <row r="182" spans="1:4">
+      <c r="E181" s="1">
+        <v>751.74</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C182" s="1">
         <v>65.98999999999999</v>
@@ -3213,10 +3759,13 @@
       <c r="D182" s="1">
         <v>510.02</v>
       </c>
-    </row>
-    <row r="183" spans="1:4">
+      <c r="E182" s="1">
+        <v>220.97</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C183" s="1">
         <v>102.98</v>
@@ -3224,21 +3773,27 @@
       <c r="D183" s="1">
         <v>887.76</v>
       </c>
-    </row>
-    <row r="184" spans="1:4">
+      <c r="E183" s="1">
+        <v>561.5300000000001</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C184" s="1">
         <v>383.13</v>
       </c>
       <c r="D184" s="1">
-        <v>848.3399999999999</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4">
+        <v>848.34</v>
+      </c>
+      <c r="E184" s="1">
+        <v>600.0799999999999</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C185" s="1">
         <v>1232.22</v>
@@ -3246,65 +3801,83 @@
       <c r="D185" s="1">
         <v>1745.88</v>
       </c>
-    </row>
-    <row r="186" spans="1:4">
+      <c r="E185" s="1">
+        <v>1090.88</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C186" s="1">
-        <v>620.87</v>
+        <v>620.8699999999999</v>
       </c>
       <c r="D186" s="1">
-        <v>706.8799999999999</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4">
+        <v>706.88</v>
+      </c>
+      <c r="E186" s="1">
+        <v>992.2</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C187" s="1">
-        <v>800.2099999999999</v>
+        <v>800.21</v>
       </c>
       <c r="D187" s="1">
         <v>500.26</v>
       </c>
-    </row>
-    <row r="188" spans="1:4">
+      <c r="E187" s="1">
+        <v>1177.45</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C188" s="1">
         <v>3277.609999999999</v>
       </c>
       <c r="D188" s="1">
-        <v>4046.089999999999</v>
-      </c>
-    </row>
-    <row r="189" spans="1:4">
+        <v>4046.09</v>
+      </c>
+      <c r="E188" s="1">
+        <v>4180.249999999999</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C189" s="1">
         <v>866.6900000000001</v>
       </c>
       <c r="D189" s="1">
-        <v>699.1099999999999</v>
-      </c>
-    </row>
-    <row r="190" spans="1:4">
+        <v>699.11</v>
+      </c>
+      <c r="E189" s="1">
+        <v>1026.66</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D190" s="1">
         <v>425.98</v>
       </c>
-    </row>
-    <row r="191" spans="1:4">
+      <c r="E190" s="1">
+        <v>263.7</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C191" s="1">
         <v>607.4</v>
@@ -3312,10 +3885,13 @@
       <c r="D191" s="1">
         <v>275.99</v>
       </c>
-    </row>
-    <row r="192" spans="1:4">
+      <c r="E191" s="1">
+        <v>395.26</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C192" s="1">
         <v>340.77</v>
@@ -3323,10 +3899,13 @@
       <c r="D192" s="1">
         <v>800</v>
       </c>
-    </row>
-    <row r="193" spans="1:4">
+      <c r="E192" s="1">
+        <v>1448.98</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C193" s="1">
         <v>648.6900000000001</v>
@@ -3334,21 +3913,27 @@
       <c r="D193" s="1">
         <v>1340.63</v>
       </c>
-    </row>
-    <row r="194" spans="1:4">
+      <c r="E193" s="1">
+        <v>1212.05</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C194" s="1">
-        <v>2649.13</v>
+        <v>2649.129999999999</v>
       </c>
       <c r="D194" s="1">
         <v>2041.4</v>
       </c>
-    </row>
-    <row r="195" spans="1:4">
+      <c r="E194" s="1">
+        <v>1552.63</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C195" s="1">
         <v>704.55</v>
@@ -3356,21 +3941,27 @@
       <c r="D195" s="1">
         <v>2509.8</v>
       </c>
-    </row>
-    <row r="196" spans="1:4">
+      <c r="E195" s="1">
+        <v>2709.7</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C196" s="1">
         <v>202.42</v>
       </c>
       <c r="D196" s="1">
-        <v>376.8200000000001</v>
-      </c>
-    </row>
-    <row r="197" spans="1:4">
+        <v>376.82</v>
+      </c>
+      <c r="E196" s="1">
+        <v>120.7</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C197" s="1">
         <v>2436.17</v>
@@ -3378,21 +3969,27 @@
       <c r="D197" s="1">
         <v>583.25</v>
       </c>
-    </row>
-    <row r="198" spans="1:4">
+      <c r="E197" s="1">
+        <v>841.86</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C198" s="1">
-        <v>859.6</v>
+        <v>859.5999999999999</v>
       </c>
       <c r="D198" s="1">
         <v>1110.7</v>
       </c>
-    </row>
-    <row r="199" spans="1:4">
+      <c r="E198" s="1">
+        <v>890.66</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C199" s="1">
         <v>428.81</v>
@@ -3400,32 +3997,41 @@
       <c r="D199" s="1">
         <v>265.14</v>
       </c>
-    </row>
-    <row r="200" spans="1:4">
+      <c r="E199" s="1">
+        <v>747.63</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D200" s="1">
         <v>86.44</v>
       </c>
-    </row>
-    <row r="201" spans="1:4">
+      <c r="E200" s="1">
+        <v>292.87</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C201" s="1">
         <v>1441.84</v>
       </c>
       <c r="D201" s="1">
-        <v>2928.27</v>
-      </c>
-    </row>
-    <row r="202" spans="1:4">
+        <v>2971.26</v>
+      </c>
+      <c r="E201" s="1">
+        <v>1711.76</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C202" s="1">
         <v>606.35</v>
@@ -3433,21 +4039,27 @@
       <c r="D202" s="1">
         <v>969.3099999999999</v>
       </c>
-    </row>
-    <row r="203" spans="1:4">
+      <c r="E202" s="1">
+        <v>244.97</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5">
       <c r="A203" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D203" s="1">
-        <v>288.94</v>
-      </c>
-    </row>
-    <row r="204" spans="1:4">
+        <v>288.9399999999999</v>
+      </c>
+      <c r="E203" s="1">
+        <v>55.99</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5">
       <c r="A204" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C204" s="1">
         <v>147.98</v>
@@ -3455,21 +4067,27 @@
       <c r="D204" s="1">
         <v>117.99</v>
       </c>
-    </row>
-    <row r="205" spans="1:4">
+      <c r="E204" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5">
       <c r="A205" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C205" s="1">
         <v>65.98999999999999</v>
       </c>
       <c r="D205" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="206" spans="1:4">
+        <v>56</v>
+      </c>
+      <c r="E205" s="1">
+        <v>557.5</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5">
       <c r="A206" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C206" s="1">
         <v>1049.99</v>
@@ -3477,10 +4095,13 @@
       <c r="D206" s="1">
         <v>472.15</v>
       </c>
-    </row>
-    <row r="207" spans="1:4">
+      <c r="E206" s="1">
+        <v>313.69</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5">
       <c r="A207" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C207" s="1">
         <v>1156.74</v>
@@ -3488,10 +4109,13 @@
       <c r="D207" s="1">
         <v>153.98</v>
       </c>
-    </row>
-    <row r="208" spans="1:4">
+      <c r="E207" s="1">
+        <v>472.6799999999999</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5">
       <c r="A208" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C208" s="1">
         <v>618.88</v>
@@ -3499,10 +4123,13 @@
       <c r="D208" s="1">
         <v>906.9400000000001</v>
       </c>
-    </row>
-    <row r="209" spans="1:4">
+      <c r="E208" s="1">
+        <v>611.91</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5">
       <c r="A209" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C209" s="1">
         <v>94.47999999999999</v>
@@ -3510,10 +4137,13 @@
       <c r="D209" s="1">
         <v>320.96</v>
       </c>
-    </row>
-    <row r="210" spans="1:4">
+      <c r="E209" s="1">
+        <v>301.38</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5">
       <c r="A210" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C210" s="1">
         <v>388.97</v>
@@ -3521,10 +4151,13 @@
       <c r="D210" s="1">
         <v>365.78</v>
       </c>
-    </row>
-    <row r="211" spans="1:4">
+      <c r="E210" s="1">
+        <v>782.65</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5">
       <c r="A211" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C211" s="1">
         <v>117.99</v>
@@ -3532,10 +4165,13 @@
       <c r="D211" s="1">
         <v>347.85</v>
       </c>
-    </row>
-    <row r="212" spans="1:4">
+      <c r="E211" s="1">
+        <v>1338.12</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5">
       <c r="A212" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C212" s="1">
         <v>449.42</v>
@@ -3543,10 +4179,13 @@
       <c r="D212" s="1">
         <v>1031.77</v>
       </c>
-    </row>
-    <row r="213" spans="1:4">
+      <c r="E212" s="1">
+        <v>700.52</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5">
       <c r="A213" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C213" s="1">
         <v>883.9299999999999</v>
@@ -3554,21 +4193,27 @@
       <c r="D213" s="1">
         <v>182.98</v>
       </c>
-    </row>
-    <row r="214" spans="1:4">
+      <c r="E213" s="1">
+        <v>1523.92</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5">
       <c r="A214" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C214" s="1">
         <v>198.22</v>
       </c>
       <c r="D214" s="1">
-        <v>377.9499999999999</v>
-      </c>
-    </row>
-    <row r="215" spans="1:4">
+        <v>377.95</v>
+      </c>
+      <c r="E214" s="1">
+        <v>474.33</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5">
       <c r="A215" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C215" s="1">
         <v>571.87</v>
@@ -3576,10 +4221,13 @@
       <c r="D215" s="1">
         <v>910.6799999999999</v>
       </c>
-    </row>
-    <row r="216" spans="1:4">
+      <c r="E215" s="1">
+        <v>373.59</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5">
       <c r="A216" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C216" s="1">
         <v>857.4299999999999</v>
@@ -3587,21 +4235,27 @@
       <c r="D216" s="1">
         <v>64.48999999999999</v>
       </c>
-    </row>
-    <row r="217" spans="1:4">
+      <c r="E216" s="1">
+        <v>439.21</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5">
       <c r="A217" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C217" s="1">
         <v>533.61</v>
       </c>
       <c r="D217" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="218" spans="1:4">
+        <v>56</v>
+      </c>
+      <c r="E217" s="1">
+        <v>707.53</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5">
       <c r="A218" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C218" s="1">
         <v>292.42</v>
@@ -3609,10 +4263,13 @@
       <c r="D218" s="1">
         <v>1025.67</v>
       </c>
-    </row>
-    <row r="219" spans="1:4">
+      <c r="E218" s="1">
+        <v>164.73</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5">
       <c r="A219" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C219" s="1">
         <v>379.26</v>
@@ -3620,10 +4277,13 @@
       <c r="D219" s="1">
         <v>456.67</v>
       </c>
-    </row>
-    <row r="220" spans="1:4">
+      <c r="E219" s="1">
+        <v>350.01</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5">
       <c r="A220" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C220" s="1">
         <v>487.18</v>
@@ -3631,10 +4291,13 @@
       <c r="D220" s="1">
         <v>199.88</v>
       </c>
-    </row>
-    <row r="221" spans="1:4">
+      <c r="E220" s="1">
+        <v>87.5</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5">
       <c r="A221" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C221" s="1">
         <v>601.58</v>
@@ -3642,21 +4305,27 @@
       <c r="D221" s="1">
         <v>64.54000000000001</v>
       </c>
-    </row>
-    <row r="222" spans="1:4">
+      <c r="E221" s="1">
+        <v>1402.61</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5">
       <c r="A222" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C222" s="1">
-        <v>837.9999999999999</v>
+        <v>838</v>
       </c>
       <c r="D222" s="1">
         <v>1258.16</v>
       </c>
-    </row>
-    <row r="223" spans="1:4">
+      <c r="E222" s="1">
+        <v>613.37</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5">
       <c r="A223" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C223" s="1">
         <v>476.16</v>
@@ -3664,10 +4333,13 @@
       <c r="D223" s="1">
         <v>897.11</v>
       </c>
-    </row>
-    <row r="224" spans="1:4">
+      <c r="E223" s="1">
+        <v>790.53</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5">
       <c r="A224" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C224" s="1">
         <v>726.36</v>
@@ -3675,10 +4347,13 @@
       <c r="D224" s="1">
         <v>1188.02</v>
       </c>
-    </row>
-    <row r="225" spans="1:4">
+      <c r="E224" s="1">
+        <v>609.59</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5">
       <c r="A225" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C225" s="1">
         <v>505.87</v>
@@ -3686,10 +4361,13 @@
       <c r="D225" s="1">
         <v>42.99000000000001</v>
       </c>
-    </row>
-    <row r="226" spans="1:4">
+      <c r="E225" s="1">
+        <v>980.26</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5">
       <c r="A226" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C226" s="1">
         <v>384.96</v>
@@ -3697,10 +4375,13 @@
       <c r="D226" s="1">
         <v>106.98</v>
       </c>
-    </row>
-    <row r="227" spans="1:4">
+      <c r="E226" s="1">
+        <v>696.8900000000001</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5">
       <c r="A227" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C227" s="1">
         <v>1453.45</v>
@@ -3708,10 +4389,13 @@
       <c r="D227" s="1">
         <v>1493.22</v>
       </c>
-    </row>
-    <row r="228" spans="1:4">
+      <c r="E227" s="1">
+        <v>2221.96</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5">
       <c r="A228" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C228" s="1">
         <v>288.53</v>
@@ -3719,10 +4403,13 @@
       <c r="D228" s="1">
         <v>153.98</v>
       </c>
-    </row>
-    <row r="229" spans="1:4">
+      <c r="E228" s="1">
+        <v>297.17</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5">
       <c r="A229" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C229" s="1">
         <v>248.25</v>
@@ -3730,10 +4417,13 @@
       <c r="D229" s="1">
         <v>220.98</v>
       </c>
-    </row>
-    <row r="230" spans="1:4">
+      <c r="E229" s="1">
+        <v>177.98</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5">
       <c r="A230" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C230" s="1">
         <v>429.44</v>
@@ -3741,10 +4431,13 @@
       <c r="D230" s="1">
         <v>1071.16</v>
       </c>
-    </row>
-    <row r="231" spans="1:4">
+      <c r="E230" s="1">
+        <v>286.97</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5">
       <c r="A231" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C231" s="1">
         <v>860.8099999999999</v>
@@ -3752,21 +4445,27 @@
       <c r="D231" s="1">
         <v>-238.49</v>
       </c>
-    </row>
-    <row r="232" spans="1:4">
+      <c r="E231" s="1">
+        <v>516.8199999999999</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5">
       <c r="A232" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C232" s="1">
         <v>102.99</v>
       </c>
       <c r="D232" s="1">
-        <v>660.47</v>
-      </c>
-    </row>
-    <row r="233" spans="1:4">
+        <v>660.4699999999999</v>
+      </c>
+      <c r="E232" s="1">
+        <v>723.21</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5">
       <c r="A233" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C233" s="1">
         <v>1203.73</v>
@@ -3774,10 +4473,13 @@
       <c r="D233" s="1">
         <v>223.21</v>
       </c>
-    </row>
-    <row r="234" spans="1:4">
+      <c r="E233" s="1">
+        <v>679.5599999999999</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5">
       <c r="A234" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C234" s="1">
         <v>619.04</v>
@@ -3785,21 +4487,27 @@
       <c r="D234" s="1">
         <v>1716.47</v>
       </c>
-    </row>
-    <row r="235" spans="1:4">
+      <c r="E234" s="1">
+        <v>644.92</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5">
       <c r="A235" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C235" s="1">
         <v>789.1700000000001</v>
       </c>
       <c r="D235" s="1">
-        <v>901.96</v>
-      </c>
-    </row>
-    <row r="236" spans="1:4">
+        <v>901.9599999999999</v>
+      </c>
+      <c r="E235" s="1">
+        <v>270.11</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5">
       <c r="A236" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C236" s="1">
         <v>691.87</v>
@@ -3807,10 +4515,13 @@
       <c r="D236" s="1">
         <v>1399.21</v>
       </c>
-    </row>
-    <row r="237" spans="1:4">
+      <c r="E236" s="1">
+        <v>1579.63</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5">
       <c r="A237" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C237" s="1">
         <v>1066.32</v>
@@ -3818,21 +4529,27 @@
       <c r="D237" s="1">
         <v>695.08</v>
       </c>
-    </row>
-    <row r="238" spans="1:4">
+      <c r="E237" s="1">
+        <v>1758.46</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5">
       <c r="A238" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C238" s="1">
         <v>446.16</v>
       </c>
       <c r="D238" s="1">
-        <v>578.1400000000001</v>
-      </c>
-    </row>
-    <row r="239" spans="1:4">
+        <v>578.14</v>
+      </c>
+      <c r="E238" s="1">
+        <v>412.6500000000001</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5">
       <c r="A239" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C239" s="1">
         <v>251.74</v>
@@ -3840,21 +4557,27 @@
       <c r="D239" s="1">
         <v>886.97</v>
       </c>
-    </row>
-    <row r="240" spans="1:4">
+      <c r="E239" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5">
       <c r="A240" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C240" s="1">
-        <v>974.6200000000001</v>
+        <v>974.62</v>
       </c>
       <c r="D240" s="1">
         <v>426.94</v>
       </c>
-    </row>
-    <row r="241" spans="1:4">
+      <c r="E240" s="1">
+        <v>888.3200000000001</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5">
       <c r="A241" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C241" s="1">
         <v>885.5599999999999</v>
@@ -3862,21 +4585,27 @@
       <c r="D241" s="1">
         <v>1253.79</v>
       </c>
-    </row>
-    <row r="242" spans="1:4">
+      <c r="E241" s="1">
+        <v>1112.32</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5">
       <c r="A242" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C242" s="1">
-        <v>3109.989999999999</v>
+        <v>3109.99</v>
       </c>
       <c r="D242" s="1">
-        <v>2529.459999999999</v>
-      </c>
-    </row>
-    <row r="243" spans="1:4">
+        <v>2529.46</v>
+      </c>
+      <c r="E242" s="1">
+        <v>1594.76</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5">
       <c r="A243" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C243" s="1">
         <v>1197.26</v>
@@ -3884,10 +4613,13 @@
       <c r="D243" s="1">
         <v>1776.03</v>
       </c>
-    </row>
-    <row r="244" spans="1:4">
+      <c r="E243" s="1">
+        <v>527.5699999999999</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5">
       <c r="A244" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C244" s="1">
         <v>912.5</v>
@@ -3895,10 +4627,13 @@
       <c r="D244" s="1">
         <v>126.98</v>
       </c>
-    </row>
-    <row r="245" spans="1:4">
+      <c r="E244" s="1">
+        <v>752.9200000000001</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5">
       <c r="A245" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C245" s="1">
         <v>1247.88</v>
@@ -3906,10 +4641,13 @@
       <c r="D245" s="1">
         <v>1219.3</v>
       </c>
-    </row>
-    <row r="246" spans="1:4">
+      <c r="E245" s="1">
+        <v>814.6400000000001</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5">
       <c r="A246" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C246" s="1">
         <v>419.26</v>
@@ -3917,21 +4655,27 @@
       <c r="D246" s="1">
         <v>2877.41</v>
       </c>
-    </row>
-    <row r="247" spans="1:4">
+      <c r="E246" s="1">
+        <v>1614.56</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5">
       <c r="A247" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C247" s="1">
-        <v>838.1199999999999</v>
+        <v>838.12</v>
       </c>
       <c r="D247" s="1">
         <v>617.7</v>
       </c>
-    </row>
-    <row r="248" spans="1:4">
+      <c r="E247" s="1">
+        <v>127.38</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5">
       <c r="A248" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C248" s="1">
         <v>1460.33</v>
@@ -3939,10 +4683,13 @@
       <c r="D248" s="1">
         <v>2472.57</v>
       </c>
-    </row>
-    <row r="249" spans="1:4">
+      <c r="E248" s="1">
+        <v>2993.779999999999</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5">
       <c r="A249" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C249" s="1">
         <v>589.9</v>
@@ -3950,21 +4697,27 @@
       <c r="D249" s="1">
         <v>689.38</v>
       </c>
-    </row>
-    <row r="250" spans="1:4">
+      <c r="E249" s="1">
+        <v>218.72</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5">
       <c r="A250" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C250" s="1">
         <v>1920.76</v>
       </c>
       <c r="D250" s="1">
-        <v>2720.139999999999</v>
-      </c>
-    </row>
-    <row r="251" spans="1:4">
+        <v>2720.14</v>
+      </c>
+      <c r="E250" s="1">
+        <v>2139.15</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5">
       <c r="A251" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C251" s="1">
         <v>222.93</v>
@@ -3972,21 +4725,27 @@
       <c r="D251" s="1">
         <v>963.5599999999999</v>
       </c>
-    </row>
-    <row r="252" spans="1:4">
+      <c r="E251" s="1">
+        <v>128.98</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5">
       <c r="A252" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C252" s="1">
         <v>296.55</v>
       </c>
       <c r="D252" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="253" spans="1:4">
+        <v>56</v>
+      </c>
+      <c r="E252" s="1">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5">
       <c r="A253" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C253" s="1">
         <v>407.72</v>
@@ -3994,21 +4753,27 @@
       <c r="D253" s="1">
         <v>274.95</v>
       </c>
-    </row>
-    <row r="254" spans="1:4">
+      <c r="E253" s="1">
+        <v>684.16</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5">
       <c r="A254" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C254" s="1">
-        <v>302.6800000000001</v>
+        <v>302.68</v>
       </c>
       <c r="D254" s="1">
-        <v>468.9499999999999</v>
-      </c>
-    </row>
-    <row r="255" spans="1:4">
+        <v>468.95</v>
+      </c>
+      <c r="E254" s="1">
+        <v>601.5</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5">
       <c r="A255" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C255" s="1">
         <v>1526.43</v>
@@ -4016,10 +4781,13 @@
       <c r="D255" s="1">
         <v>1758.1</v>
       </c>
-    </row>
-    <row r="256" spans="1:4">
+      <c r="E255" s="1">
+        <v>1445.09</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5">
       <c r="A256" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C256" s="1">
         <v>166.89</v>
@@ -4027,10 +4795,13 @@
       <c r="D256" s="1">
         <v>140.19</v>
       </c>
-    </row>
-    <row r="257" spans="1:4">
+      <c r="E256" s="1">
+        <v>42.99</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5">
       <c r="A257" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C257" s="1">
         <v>1067.2</v>
@@ -4038,10 +4809,13 @@
       <c r="D257" s="1">
         <v>1214.39</v>
       </c>
-    </row>
-    <row r="258" spans="1:4">
+      <c r="E257" s="1">
+        <v>713.8200000000001</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5">
       <c r="A258" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C258" s="1">
         <v>414.1500000000001</v>
@@ -4049,21 +4823,27 @@
       <c r="D258" s="1">
         <v>92.84999999999999</v>
       </c>
-    </row>
-    <row r="259" spans="1:4">
+      <c r="E258" s="1">
+        <v>255.07</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5">
       <c r="A259" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C259" s="1">
         <v>1089.29</v>
       </c>
       <c r="D259" s="1">
-        <v>646.5500000000002</v>
-      </c>
-    </row>
-    <row r="260" spans="1:4">
+        <v>646.55</v>
+      </c>
+      <c r="E259" s="1">
+        <v>1627.83</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5">
       <c r="A260" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C260" s="1">
         <v>1477.84</v>
@@ -4071,10 +4851,13 @@
       <c r="D260" s="1">
         <v>1394.24</v>
       </c>
-    </row>
-    <row r="261" spans="1:4">
+      <c r="E260" s="1">
+        <v>841.21</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5">
       <c r="A261" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C261" s="1">
         <v>630.26</v>
@@ -4082,10 +4865,13 @@
       <c r="D261" s="1">
         <v>470.98</v>
       </c>
-    </row>
-    <row r="262" spans="1:4">
+      <c r="E261" s="1">
+        <v>212.38</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5">
       <c r="A262" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C262" s="1">
         <v>2722.72</v>
@@ -4093,10 +4879,13 @@
       <c r="D262" s="1">
         <v>1228.43</v>
       </c>
-    </row>
-    <row r="263" spans="1:4">
+      <c r="E262" s="1">
+        <v>1594.58</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5">
       <c r="A263" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C263" s="1">
         <v>1131.02</v>
@@ -4104,10 +4893,13 @@
       <c r="D263" s="1">
         <v>768.8200000000001</v>
       </c>
-    </row>
-    <row r="264" spans="1:4">
+      <c r="E263" s="1">
+        <v>1001.11</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5">
       <c r="A264" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C264" s="1">
         <v>648.9400000000001</v>
@@ -4115,10 +4907,13 @@
       <c r="D264" s="1">
         <v>460.85</v>
       </c>
-    </row>
-    <row r="265" spans="1:4">
+      <c r="E264" s="1">
+        <v>494.0699999999999</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5">
       <c r="A265" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C265" s="1">
         <v>2099.16</v>
@@ -4126,10 +4921,13 @@
       <c r="D265" s="1">
         <v>1972.77</v>
       </c>
-    </row>
-    <row r="266" spans="1:4">
+      <c r="E265" s="1">
+        <v>1095.34</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5">
       <c r="A266" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C266" s="1">
         <v>1077.83</v>
@@ -4137,10 +4935,13 @@
       <c r="D266" s="1">
         <v>1839.39</v>
       </c>
-    </row>
-    <row r="267" spans="1:4">
+      <c r="E266" s="1">
+        <v>566.25</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5">
       <c r="A267" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C267" s="1">
         <v>2945.049999999999</v>
@@ -4148,10 +4949,13 @@
       <c r="D267" s="1">
         <v>1387.05</v>
       </c>
-    </row>
-    <row r="268" spans="1:4">
+      <c r="E267" s="1">
+        <v>669.48</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5">
       <c r="A268" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C268" s="1">
         <v>517.67</v>
@@ -4159,10 +4963,13 @@
       <c r="D268" s="1">
         <v>833.55</v>
       </c>
-    </row>
-    <row r="269" spans="1:4">
+      <c r="E268" s="1">
+        <v>357.32</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5">
       <c r="A269" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C269" s="1">
         <v>142.12</v>
@@ -4170,16 +4977,22 @@
       <c r="D269" s="1">
         <v>167.29</v>
       </c>
-    </row>
-    <row r="270" spans="1:4">
+      <c r="E269" s="1">
+        <v>228.63</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5">
       <c r="A270" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C270" s="1">
         <v>241.74</v>
       </c>
       <c r="D270" s="1">
         <v>331.72</v>
+      </c>
+      <c r="E270" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>